<commit_message>
Ayar karşılaştırması ve zorlaştırılmış örnek soru seti
- ayar_karsilastir.sh / python -m degerlendirme.karsilastir: parça boyutu,
  top_k ve cevap modelini her seferinde tek tek değiştirerek değerlendirmeyi
  tekrarlar; tek karşılaştırma tablosu (karsilastirma.xlsx) ve öneri üretir.
  Her denemede aynı hakem ve temiz veri klasörü; önerilen birleşim daha önce
  denenmediyse ayrıca doğrulanır; eksik modeller (disk kontrolüyle) indirilir.
- Öneri kuralı sıradan bağımsız: en yüksek doğruluğa bir soru mesafesindeki
  denemeler arasından algılanan beklemesi en kısa olan.
- Rapora "algılanan bekleme" (ilk kelime ya da Excel'de cevabın tamamı).
- Örnek set 14 → 24 soru: farklı kelimelerle sorulan, kural/hesap gerektiren,
  yönlendirmeyi şaşırtan ve "dokümanda olmayan" tuzak sorular.
- llm.pull(), run_evaluation() (özet döndürür), hakem sonrası bellek boşaltma.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L9wQRKfk678C1qPao26uMA
</commit_message>
<xml_diff>
--- a/ornekler/degerlendirme/sorular.xlsx
+++ b/ornekler/degerlendirme/sorular.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -774,6 +774,232 @@
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>dokümanda olmayan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>7 yıldır bu şirketteyim, yıllık kaç gün tatil hakkım var?</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>20 iş günü</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>personel_yonetmeligi.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>doküman</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Babam vefat etti; kaç gün izin alabilirim ve bu yıllık iznimden düşer mi?</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>3 gün ücretli mazeret izni; yıllık izinden düşülmez</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>personel_yonetmeligi.pdf</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>doküman</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>İşe yeni başladım, ilk ayımda evden çalışabilir miyim?</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Hayır; deneme süresindeki (2 ay) çalışanlar uzaktan çalışamaz</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>personel_yonetmeligi.pdf</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>doküman</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Ankara'ya 2 gecelik iş seyahatinde konaklamaya en fazla ne kadar harcayabilirim?</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Gecelik 3.500 TL, iki gece için toplam 7.000 TL</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>personel_yonetmeligi.pdf</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>doküman</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Hastalık raporu aldığım günlerin ücretini kim öder?</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>İlk 2 günün ücretini şirket öder</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>personel_yonetmeligi.pdf</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>doküman</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Londra'daki kahvehanelere hangi ad verilmişti ve neden?</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>'Penny üniversiteleri'; bir bardak kahve karşılığında saatlerce entelektüel tartışmalara katılmak mümkündü</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>kahve_tarihi.pdf</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>doküman</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Ankara'da Laptop satışlarından elde edilen toplam tutar nedir?</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>608.000 TL</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>satislar.xlsx</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Ocak ayından Mart ayına toplam satış tutarı arttı mı azaldı mı, ne kadar?</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>arttı: Ocak 905.500 TL, Mart 1.106.800 TL, fark 201.300 TL</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>satislar.xlsx</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Yurt dışı iş seyahatlerinde gecelik konaklama üst sınırı nedir?</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>dokümanda olmayan</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Doğum yapan bir çalışana kaç gün doğum izni verilir?</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>dokümanda olmayan</t>
         </is>

</xml_diff>